<commit_message>
first update to the sheet files
</commit_message>
<xml_diff>
--- a/CasesAFR/AFR0.8.xlsx
+++ b/CasesAFR/AFR0.8.xlsx
@@ -1,22 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\s202180910\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\afsalem\Documents\GitHub\Senior_Project_Dashboard\CasesAFR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A375CE65-20BA-49FD-ACCE-8D8BAC6F18AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{390B6B1A-B78F-4C4D-ABF2-4E3F0739C4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Energy Streams" sheetId="1" r:id="rId1"/>
-    <sheet name="Compositions" sheetId="2" r:id="rId2"/>
-    <sheet name="Material Streams" sheetId="3" r:id="rId3"/>
-    <sheet name="WorkBook Summary" sheetId="4" r:id="rId4"/>
+    <sheet name="Compositions" sheetId="2" r:id="rId1"/>
+    <sheet name="Material Streams" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -28,17 +26,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="37">
   <si>
     <t>Unit</t>
   </si>
   <si>
-    <t>Heat Duty</t>
-  </si>
-  <si>
-    <t>WTurbine</t>
-  </si>
-  <si>
     <t>Heat Flow</t>
   </si>
   <si>
@@ -145,27 +137,12 @@
   </si>
   <si>
     <t>m3/h</t>
-  </si>
-  <si>
-    <t>Case:</t>
-  </si>
-  <si>
-    <t>c:\Users\s202180910\AppData\Local\Temp\be964386-ba9d-43ed-98e9-30b3f0237f7b_MeetingRelatedfile.zip.f7b\HysysCase.hsc</t>
-  </si>
-  <si>
-    <t>Flowsheet:</t>
-  </si>
-  <si>
-    <t>Main</t>
-  </si>
-  <si>
-    <t>Current Flowsheet Environment:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1033,37 +1010,508 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:K15"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="9.140625" style="1"/>
+    <col min="2" max="2" width="9.1796875" style="1"/>
+    <col min="3" max="3" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="12" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C3" s="4">
         <v>0</v>
       </c>
-      <c r="D3" s="4">
-        <v>33395718.422102768</v>
+      <c r="D3" s="1">
+        <v>1.7614892314972933E-11</v>
+      </c>
+      <c r="E3" s="1">
+        <v>1.7614892314972933E-11</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0</v>
+      </c>
+      <c r="G3" s="1">
+        <v>1.7614892314972933E-11</v>
+      </c>
+      <c r="H3" s="4">
+        <v>0.8</v>
+      </c>
+      <c r="I3" s="1">
+        <v>1.7614892314972933E-11</v>
+      </c>
+      <c r="J3" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="K3" s="1">
+        <v>1.7614892314972933E-11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="4">
+        <v>0</v>
+      </c>
+      <c r="D4" s="1">
+        <v>5.6620742769169838E-34</v>
+      </c>
+      <c r="E4" s="1">
+        <v>5.6620742769169838E-34</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0</v>
+      </c>
+      <c r="G4" s="1">
+        <v>5.6620742769169838E-34</v>
+      </c>
+      <c r="H4" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="I4" s="1">
+        <v>5.6620742769169838E-34</v>
+      </c>
+      <c r="J4" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="K4" s="1">
+        <v>5.6620742769169838E-34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="4">
+        <v>0</v>
+      </c>
+      <c r="D5" s="1">
+        <v>3.7959950171632794E-39</v>
+      </c>
+      <c r="E5" s="1">
+        <v>3.7959950171632794E-39</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0</v>
+      </c>
+      <c r="G5" s="1">
+        <v>3.7959950171632794E-39</v>
+      </c>
+      <c r="H5" s="4">
+        <v>0.02</v>
+      </c>
+      <c r="I5" s="1">
+        <v>3.7959950171632794E-39</v>
+      </c>
+      <c r="J5" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="K5" s="1">
+        <v>3.7959950171632794E-39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="4">
+        <v>0</v>
+      </c>
+      <c r="D6" s="1">
+        <v>3.461928029971746E-39</v>
+      </c>
+      <c r="E6" s="1">
+        <v>3.461928029971746E-39</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0</v>
+      </c>
+      <c r="G6" s="1">
+        <v>3.461928029971746E-39</v>
+      </c>
+      <c r="H6" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="I6" s="1">
+        <v>3.461928029971746E-39</v>
+      </c>
+      <c r="J6" s="1">
+        <v>0.01</v>
+      </c>
+      <c r="K6" s="1">
+        <v>3.461928029971746E-39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="4">
+        <v>0</v>
+      </c>
+      <c r="D7" s="1">
+        <v>3.6626503554407977E-23</v>
+      </c>
+      <c r="E7" s="1">
+        <v>3.6626503554407977E-23</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0</v>
+      </c>
+      <c r="G7" s="1">
+        <v>3.6626503554407977E-23</v>
+      </c>
+      <c r="H7" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="I7" s="1">
+        <v>3.6626503554407977E-23</v>
+      </c>
+      <c r="J7" s="1">
+        <v>0.05</v>
+      </c>
+      <c r="K7" s="1">
+        <v>3.6626503554407977E-23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="4">
+        <v>0</v>
+      </c>
+      <c r="D8" s="1">
+        <v>5.7320448295746368E-2</v>
+      </c>
+      <c r="E8" s="1">
+        <v>5.7320448295746368E-2</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0</v>
+      </c>
+      <c r="G8" s="1">
+        <v>5.7320448295746368E-2</v>
+      </c>
+      <c r="H8" s="4">
+        <v>0</v>
+      </c>
+      <c r="I8" s="1">
+        <v>5.7320448295746368E-2</v>
+      </c>
+      <c r="J8" s="1">
+        <v>0</v>
+      </c>
+      <c r="K8" s="1">
+        <v>5.7320448295746368E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="4">
+        <v>0</v>
+      </c>
+      <c r="D9" s="1">
+        <v>6.2279834516033569E-2</v>
+      </c>
+      <c r="E9" s="1">
+        <v>6.2279834516033569E-2</v>
+      </c>
+      <c r="F9" s="1">
+        <v>0</v>
+      </c>
+      <c r="G9" s="1">
+        <v>6.2279834516033569E-2</v>
+      </c>
+      <c r="H9" s="4">
+        <v>0</v>
+      </c>
+      <c r="I9" s="1">
+        <v>6.2279834516033569E-2</v>
+      </c>
+      <c r="J9" s="1">
+        <v>0</v>
+      </c>
+      <c r="K9" s="1">
+        <v>6.2279834516033569E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="4">
+        <v>0</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0.17510399197318455</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0.17510399197318455</v>
+      </c>
+      <c r="F10" s="1">
+        <v>0</v>
+      </c>
+      <c r="G10" s="1">
+        <v>0.17510399197318455</v>
+      </c>
+      <c r="H10" s="4">
+        <v>0</v>
+      </c>
+      <c r="I10" s="1">
+        <v>0.17510399197318455</v>
+      </c>
+      <c r="J10" s="1">
+        <v>0</v>
+      </c>
+      <c r="K10" s="1">
+        <v>0.17510399197318455</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="4">
+        <v>0</v>
+      </c>
+      <c r="D11" s="1">
+        <v>3.3750233230976381E-2</v>
+      </c>
+      <c r="E11" s="1">
+        <v>3.3750233230976381E-2</v>
+      </c>
+      <c r="F11" s="1">
+        <v>0</v>
+      </c>
+      <c r="G11" s="1">
+        <v>3.3750233230976381E-2</v>
+      </c>
+      <c r="H11" s="4">
+        <v>0.02</v>
+      </c>
+      <c r="I11" s="1">
+        <v>3.3750233230976381E-2</v>
+      </c>
+      <c r="J11" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="K11" s="1">
+        <v>3.3750233230976381E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="4">
+        <v>0</v>
+      </c>
+      <c r="D12" s="1">
+        <v>3.1344170128357961E-10</v>
+      </c>
+      <c r="E12" s="1">
+        <v>3.1344170128357961E-10</v>
+      </c>
+      <c r="F12" s="1">
+        <v>0</v>
+      </c>
+      <c r="G12" s="1">
+        <v>3.1344170128357961E-10</v>
+      </c>
+      <c r="H12" s="4">
+        <v>0</v>
+      </c>
+      <c r="I12" s="1">
+        <v>3.1344170128357961E-10</v>
+      </c>
+      <c r="J12" s="1">
+        <v>0</v>
+      </c>
+      <c r="K12" s="1">
+        <v>3.1344170128357961E-10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="4">
+        <v>0</v>
+      </c>
+      <c r="D13" s="1">
+        <v>2.8458472535517958E-5</v>
+      </c>
+      <c r="E13" s="1">
+        <v>2.8458472535517958E-5</v>
+      </c>
+      <c r="F13" s="1">
+        <v>0</v>
+      </c>
+      <c r="G13" s="1">
+        <v>2.8458472535517958E-5</v>
+      </c>
+      <c r="H13" s="4">
+        <v>0</v>
+      </c>
+      <c r="I13" s="1">
+        <v>2.8458472535517958E-5</v>
+      </c>
+      <c r="J13" s="1">
+        <v>0</v>
+      </c>
+      <c r="K13" s="1">
+        <v>2.8458472535517958E-5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" s="4">
+        <v>0.21</v>
+      </c>
+      <c r="D14" s="1">
+        <v>1.6006222611101441E-6</v>
+      </c>
+      <c r="E14" s="1">
+        <v>1.6006222611101441E-6</v>
+      </c>
+      <c r="F14" s="1">
+        <v>0.21</v>
+      </c>
+      <c r="G14" s="1">
+        <v>1.6006222611101441E-6</v>
+      </c>
+      <c r="H14" s="4">
+        <v>0</v>
+      </c>
+      <c r="I14" s="1">
+        <v>1.6006222611101439E-6</v>
+      </c>
+      <c r="J14" s="1">
+        <v>0</v>
+      </c>
+      <c r="K14" s="1">
+        <v>1.6006222611101441E-6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="4">
+        <v>0.79</v>
+      </c>
+      <c r="D15" s="1">
+        <v>0.67151543255820589</v>
+      </c>
+      <c r="E15" s="1">
+        <v>0.67151543255820589</v>
+      </c>
+      <c r="F15" s="1">
+        <v>0.79000000000000015</v>
+      </c>
+      <c r="G15" s="1">
+        <v>0.67151543255820589</v>
+      </c>
+      <c r="H15" s="4">
+        <v>0</v>
+      </c>
+      <c r="I15" s="1">
+        <v>0.67151543255820589</v>
+      </c>
+      <c r="J15" s="1">
+        <v>0</v>
+      </c>
+      <c r="K15" s="1">
+        <v>0.67151543255820589</v>
       </c>
     </row>
   </sheetData>
@@ -1072,569 +1520,59 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" style="1"/>
-    <col min="3" max="3" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="1"/>
+    <col min="2" max="2" width="9.1796875" style="1"/>
+    <col min="3" max="3" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="11.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="J1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="K1" s="3" t="s">
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="4">
-        <v>0</v>
-      </c>
-      <c r="D3" s="1">
-        <v>1.7614892314972933E-11</v>
-      </c>
-      <c r="E3" s="1">
-        <v>1.7614892314972933E-11</v>
-      </c>
-      <c r="F3" s="1">
-        <v>0</v>
-      </c>
-      <c r="G3" s="1">
-        <v>1.7614892314972933E-11</v>
-      </c>
-      <c r="H3" s="4">
-        <v>0.8</v>
-      </c>
-      <c r="I3" s="1">
-        <v>1.7614892314972933E-11</v>
-      </c>
-      <c r="J3" s="1">
-        <v>0.8</v>
-      </c>
-      <c r="K3" s="1">
-        <v>1.7614892314972933E-11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="4">
-        <v>0</v>
-      </c>
-      <c r="D4" s="1">
-        <v>5.6620742769169838E-34</v>
-      </c>
-      <c r="E4" s="1">
-        <v>5.6620742769169838E-34</v>
-      </c>
-      <c r="F4" s="1">
-        <v>0</v>
-      </c>
-      <c r="G4" s="1">
-        <v>5.6620742769169838E-34</v>
-      </c>
-      <c r="H4" s="4">
-        <v>0.1</v>
-      </c>
-      <c r="I4" s="1">
-        <v>5.6620742769169838E-34</v>
-      </c>
-      <c r="J4" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="K4" s="1">
-        <v>5.6620742769169838E-34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="4">
-        <v>0</v>
-      </c>
-      <c r="D5" s="1">
-        <v>3.7959950171632794E-39</v>
-      </c>
-      <c r="E5" s="1">
-        <v>3.7959950171632794E-39</v>
-      </c>
-      <c r="F5" s="1">
-        <v>0</v>
-      </c>
-      <c r="G5" s="1">
-        <v>3.7959950171632794E-39</v>
-      </c>
-      <c r="H5" s="4">
-        <v>0.02</v>
-      </c>
-      <c r="I5" s="1">
-        <v>3.7959950171632794E-39</v>
-      </c>
-      <c r="J5" s="1">
-        <v>0.02</v>
-      </c>
-      <c r="K5" s="1">
-        <v>3.7959950171632794E-39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="4">
-        <v>0</v>
-      </c>
-      <c r="D6" s="1">
-        <v>3.461928029971746E-39</v>
-      </c>
-      <c r="E6" s="1">
-        <v>3.461928029971746E-39</v>
-      </c>
-      <c r="F6" s="1">
-        <v>0</v>
-      </c>
-      <c r="G6" s="1">
-        <v>3.461928029971746E-39</v>
-      </c>
-      <c r="H6" s="4">
-        <v>0.01</v>
-      </c>
-      <c r="I6" s="1">
-        <v>3.461928029971746E-39</v>
-      </c>
-      <c r="J6" s="1">
-        <v>0.01</v>
-      </c>
-      <c r="K6" s="1">
-        <v>3.461928029971746E-39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="4">
-        <v>0</v>
-      </c>
-      <c r="D7" s="1">
-        <v>3.6626503554407977E-23</v>
-      </c>
-      <c r="E7" s="1">
-        <v>3.6626503554407977E-23</v>
-      </c>
-      <c r="F7" s="1">
-        <v>0</v>
-      </c>
-      <c r="G7" s="1">
-        <v>3.6626503554407977E-23</v>
-      </c>
-      <c r="H7" s="4">
-        <v>0.05</v>
-      </c>
-      <c r="I7" s="1">
-        <v>3.6626503554407977E-23</v>
-      </c>
-      <c r="J7" s="1">
-        <v>0.05</v>
-      </c>
-      <c r="K7" s="1">
-        <v>3.6626503554407977E-23</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="4">
-        <v>0</v>
-      </c>
-      <c r="D8" s="1">
-        <v>5.7320448295746368E-2</v>
-      </c>
-      <c r="E8" s="1">
-        <v>5.7320448295746368E-2</v>
-      </c>
-      <c r="F8" s="1">
-        <v>0</v>
-      </c>
-      <c r="G8" s="1">
-        <v>5.7320448295746368E-2</v>
-      </c>
-      <c r="H8" s="4">
-        <v>0</v>
-      </c>
-      <c r="I8" s="1">
-        <v>5.7320448295746368E-2</v>
-      </c>
-      <c r="J8" s="1">
-        <v>0</v>
-      </c>
-      <c r="K8" s="1">
-        <v>5.7320448295746368E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="4">
-        <v>0</v>
-      </c>
-      <c r="D9" s="1">
-        <v>6.2279834516033569E-2</v>
-      </c>
-      <c r="E9" s="1">
-        <v>6.2279834516033569E-2</v>
-      </c>
-      <c r="F9" s="1">
-        <v>0</v>
-      </c>
-      <c r="G9" s="1">
-        <v>6.2279834516033569E-2</v>
-      </c>
-      <c r="H9" s="4">
-        <v>0</v>
-      </c>
-      <c r="I9" s="1">
-        <v>6.2279834516033569E-2</v>
-      </c>
-      <c r="J9" s="1">
-        <v>0</v>
-      </c>
-      <c r="K9" s="1">
-        <v>6.2279834516033569E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" s="4">
-        <v>0</v>
-      </c>
-      <c r="D10" s="1">
-        <v>0.17510399197318455</v>
-      </c>
-      <c r="E10" s="1">
-        <v>0.17510399197318455</v>
-      </c>
-      <c r="F10" s="1">
-        <v>0</v>
-      </c>
-      <c r="G10" s="1">
-        <v>0.17510399197318455</v>
-      </c>
-      <c r="H10" s="4">
-        <v>0</v>
-      </c>
-      <c r="I10" s="1">
-        <v>0.17510399197318455</v>
-      </c>
-      <c r="J10" s="1">
-        <v>0</v>
-      </c>
-      <c r="K10" s="1">
-        <v>0.17510399197318455</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" s="4">
-        <v>0</v>
-      </c>
-      <c r="D11" s="1">
-        <v>3.3750233230976381E-2</v>
-      </c>
-      <c r="E11" s="1">
-        <v>3.3750233230976381E-2</v>
-      </c>
-      <c r="F11" s="1">
-        <v>0</v>
-      </c>
-      <c r="G11" s="1">
-        <v>3.3750233230976381E-2</v>
-      </c>
-      <c r="H11" s="4">
-        <v>0.02</v>
-      </c>
-      <c r="I11" s="1">
-        <v>3.3750233230976381E-2</v>
-      </c>
-      <c r="J11" s="1">
-        <v>0.02</v>
-      </c>
-      <c r="K11" s="1">
-        <v>3.3750233230976381E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" s="4">
-        <v>0</v>
-      </c>
-      <c r="D12" s="1">
-        <v>3.1344170128357961E-10</v>
-      </c>
-      <c r="E12" s="1">
-        <v>3.1344170128357961E-10</v>
-      </c>
-      <c r="F12" s="1">
-        <v>0</v>
-      </c>
-      <c r="G12" s="1">
-        <v>3.1344170128357961E-10</v>
-      </c>
-      <c r="H12" s="4">
-        <v>0</v>
-      </c>
-      <c r="I12" s="1">
-        <v>3.1344170128357961E-10</v>
-      </c>
-      <c r="J12" s="1">
-        <v>0</v>
-      </c>
-      <c r="K12" s="1">
-        <v>3.1344170128357961E-10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" s="4">
-        <v>0</v>
-      </c>
-      <c r="D13" s="1">
-        <v>2.8458472535517958E-5</v>
-      </c>
-      <c r="E13" s="1">
-        <v>2.8458472535517958E-5</v>
-      </c>
-      <c r="F13" s="1">
-        <v>0</v>
-      </c>
-      <c r="G13" s="1">
-        <v>2.8458472535517958E-5</v>
-      </c>
-      <c r="H13" s="4">
-        <v>0</v>
-      </c>
-      <c r="I13" s="1">
-        <v>2.8458472535517958E-5</v>
-      </c>
-      <c r="J13" s="1">
-        <v>0</v>
-      </c>
-      <c r="K13" s="1">
-        <v>2.8458472535517958E-5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" s="4">
-        <v>0.21</v>
-      </c>
-      <c r="D14" s="1">
-        <v>1.6006222611101441E-6</v>
-      </c>
-      <c r="E14" s="1">
-        <v>1.6006222611101441E-6</v>
-      </c>
-      <c r="F14" s="1">
-        <v>0.21</v>
-      </c>
-      <c r="G14" s="1">
-        <v>1.6006222611101441E-6</v>
-      </c>
-      <c r="H14" s="4">
-        <v>0</v>
-      </c>
-      <c r="I14" s="1">
-        <v>1.6006222611101439E-6</v>
-      </c>
-      <c r="J14" s="1">
-        <v>0</v>
-      </c>
-      <c r="K14" s="1">
-        <v>1.6006222611101441E-6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15" s="4">
-        <v>0.79</v>
-      </c>
-      <c r="D15" s="1">
-        <v>0.67151543255820589</v>
-      </c>
-      <c r="E15" s="1">
-        <v>0.67151543255820589</v>
-      </c>
-      <c r="F15" s="1">
-        <v>0.79000000000000015</v>
-      </c>
-      <c r="G15" s="1">
-        <v>0.67151543255820589</v>
-      </c>
-      <c r="H15" s="4">
-        <v>0</v>
-      </c>
-      <c r="I15" s="1">
-        <v>0.67151543255820589</v>
-      </c>
-      <c r="J15" s="1">
-        <v>0</v>
-      </c>
-      <c r="K15" s="1">
-        <v>0.67151543255820589</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="21" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" style="1"/>
-    <col min="3" max="3" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="C3" s="1">
         <v>1</v>
@@ -1664,12 +1602,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C4" s="4">
         <v>40</v>
@@ -1699,12 +1637,12 @@
         <v>1591.1806697729253</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C5" s="4">
         <v>1000</v>
@@ -1734,12 +1672,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C6" s="1">
         <v>2658.7257834548823</v>
@@ -1769,12 +1707,12 @@
         <v>3119.0993373221586</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C7" s="1">
         <v>76704.957734217591</v>
@@ -1804,12 +1742,12 @@
         <v>82285.390165068864</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C8" s="1">
         <v>88.670985579215838</v>
@@ -1839,12 +1777,12 @@
         <v>102.32037090352131</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C9" s="1">
         <v>972568.40497310599</v>
@@ -1872,44 +1810,6 @@
       </c>
       <c r="K9" s="1">
         <v>-54306121.432120427</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="21" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="9.140625" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>